<commit_message>
Correcao - Parentese sem fechamento no cursor.execute em add_produto
</commit_message>
<xml_diff>
--- a/app/exports/Pesquisa_assai_2024-07-07.xlsx
+++ b/app/exports/Pesquisa_assai_2024-07-07.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,122 +469,6 @@
           <t>data</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>7891098042385</v>
-      </c>
-      <c r="B2" t="n">
-        <v>94116</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>PREP.BEB.LEAO DRINKS PESSEGO</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>20G</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1.39</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>7894900700015</v>
-      </c>
-      <c r="B3" t="n">
-        <v>40669</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>REF.COCA-COLA ZERO LATA</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>350ML</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>2.59</v>
-      </c>
-      <c r="F3" t="n">
-        <v>2.31</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2024-07-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>7896020160052</v>
-      </c>
-      <c r="B4" t="n">
-        <v>16474</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TENYS PE BARUEL PO TRAD.ORIGINAL</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>100G</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>3.95</v>
-      </c>
-      <c r="F4" t="n">
-        <v>3.52</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>atakarejo</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2024-07-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>27898286200071</v>
-      </c>
-      <c r="B5" t="n">
-        <v>22225</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CAFE MARATA ALMOFADA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>500G</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>